<commit_message>
Mozart: Aula PWM e exemplo de codigo
</commit_message>
<xml_diff>
--- a/Exemplos_Codigo_STM32/calculoTimer.xlsx
+++ b/Exemplos_Codigo_STM32/calculoTimer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\GIT_AULAS_FATEC\Exemplos_Codigo_STM32\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2384EBDF-9A70-46B6-B978-16D3F72476D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0D5D98C-E2A4-4468-B453-EA518DF69E24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0F553953-7539-41EE-9D73-D6F519E96D34}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0F553953-7539-41EE-9D73-D6F519E96D34}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -236,22 +236,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -259,6 +254,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -593,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{432F2CC5-A964-4EB5-A8D8-F3E958E3BF7D}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
@@ -614,21 +612,21 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <v>72</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="9">
         <f>B3*1000000</f>
         <v>72000000</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="15">
-        <v>1.4999999999999999E-2</v>
+      <c r="F3" s="12">
+        <v>0.01</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -636,15 +634,14 @@
         <v>1</v>
       </c>
       <c r="B4" s="2">
-        <v>1</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="E4" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="13">
+      <c r="F4" s="10">
         <f>F3/B6</f>
-        <v>1080000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -652,9 +649,8 @@
         <v>9</v>
       </c>
       <c r="B5" s="2">
-        <v>65535</v>
-      </c>
-      <c r="C5" s="3"/>
+        <v>1000</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -662,75 +658,33 @@
       </c>
       <c r="B6" s="2">
         <f>1/(C3/B4)</f>
-        <v>1.3888888888888889E-8</v>
-      </c>
-      <c r="C6" s="3"/>
+        <v>9.9999999999999995E-7</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="2">
         <f>B6*B5</f>
-        <v>9.1020833333333329E-4</v>
-      </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+        <v>1E-3</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="8">
         <f>1/B7</f>
-        <v>1098.6495765621423</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
+        <v>1000</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Mozart: Aula Sonda LAmbda e exemplos de código
</commit_message>
<xml_diff>
--- a/Exemplos_Codigo_STM32/calculoTimer.xlsx
+++ b/Exemplos_Codigo_STM32/calculoTimer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\GIT_AULAS_FATEC\Exemplos_Codigo_STM32\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0D5D98C-E2A4-4468-B453-EA518DF69E24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0558DB17-D31F-4BE5-843B-6C940CF9E37A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0F553953-7539-41EE-9D73-D6F519E96D34}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0F553953-7539-41EE-9D73-D6F519E96D34}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>

</xml_diff>